<commit_message>
fix(charts): align degree-day metrics to active season and eliminate synthetic noise from historical matrices
</commit_message>
<xml_diff>
--- a/outputs/historical_hdd_thresholds.xlsx
+++ b/outputs/historical_hdd_thresholds.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDD Matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -650,19 +650,19 @@
         <v>30</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>30</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>30</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>30</v>
@@ -674,10 +674,10 @@
         <v>30</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="N4" s="5" t="n">
         <v>30</v>
@@ -707,16 +707,16 @@
         <v>30</v>
       </c>
       <c r="W4" s="5" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="X4" s="5" t="n">
         <v>30</v>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Z4" s="5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -967,10 +967,10 @@
         <v>31</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>31</v>
@@ -1009,7 +1009,7 @@
         <v>31</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="R8" s="5" t="n">
         <v>31</v>
@@ -1024,10 +1024,10 @@
         <v>31</v>
       </c>
       <c r="V8" s="5" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="W8" s="5" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="X8" s="5" t="n">
         <v>31</v>
@@ -1049,22 +1049,22 @@
         <v>151</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>152</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>151</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>152</v>
@@ -1076,10 +1076,10 @@
         <v>151</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="N9" s="7" t="n">
         <v>151</v>
@@ -1091,7 +1091,7 @@
         <v>151</v>
       </c>
       <c r="Q9" s="7" t="n">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="R9" s="7" t="n">
         <v>151</v>
@@ -1106,19 +1106,19 @@
         <v>152</v>
       </c>
       <c r="V9" s="7" t="n">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="W9" s="7" t="n">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>152</v>
       </c>
       <c r="Y9" s="7" t="n">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Z9" s="7" t="n">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10">
@@ -1131,22 +1131,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>1</v>
+        <v>0.9867549668874173</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>1</v>
+        <v>0.9735099337748344</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>1</v>
+        <v>0.9867549668874173</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>1</v>
+        <v>0.9735099337748344</v>
       </c>
       <c r="I10" s="8" t="n">
         <v>1</v>
@@ -1158,10 +1158,10 @@
         <v>1</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>1</v>
+        <v>0.9867549668874173</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>1</v>
+        <v>0.9802631578947368</v>
       </c>
       <c r="N10" s="8" t="n">
         <v>1</v>
@@ -1173,7 +1173,7 @@
         <v>1</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>1</v>
+        <v>0.9671052631578947</v>
       </c>
       <c r="R10" s="8" t="n">
         <v>1</v>
@@ -1188,19 +1188,19 @@
         <v>1</v>
       </c>
       <c r="V10" s="8" t="n">
-        <v>1</v>
+        <v>0.9933774834437086</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>1</v>
+        <v>0.9735099337748344</v>
       </c>
       <c r="X10" s="8" t="n">
         <v>1.006622516556291</v>
       </c>
       <c r="Y10" s="8" t="n">
-        <v>1.001324503311258</v>
+        <v>0.9920529801324504</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>1.00157678965626</v>
+        <v>0.9943235572374645</v>
       </c>
     </row>
     <row r="13">
@@ -1210,79 +1210,79 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>-31</v>
+        <v>0</v>
       </c>
       <c r="C13" s="10" t="n">
-        <v>49</v>
+        <v>-365</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>7</v>
+        <v>-452</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>57</v>
+        <v>-751</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>-67</v>
+        <v>-618</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>-56</v>
+        <v>-403</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>17</v>
+        <v>-469</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>79</v>
+        <v>-553</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>-33</v>
+        <v>-92</v>
       </c>
       <c r="K13" s="10" t="n">
-        <v>29</v>
+        <v>-185</v>
       </c>
       <c r="L13" s="10" t="n">
-        <v>-20</v>
+        <v>-705</v>
       </c>
       <c r="M13" s="10" t="n">
-        <v>-56</v>
+        <v>-874</v>
       </c>
       <c r="N13" s="10" t="n">
-        <v>63</v>
+        <v>235</v>
       </c>
       <c r="O13" s="10" t="n">
-        <v>-17</v>
+        <v>411</v>
       </c>
       <c r="P13" s="10" t="n">
-        <v>62</v>
+        <v>-236</v>
       </c>
       <c r="Q13" s="10" t="n">
-        <v>-98</v>
+        <v>-995</v>
       </c>
       <c r="R13" s="10" t="n">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="S13" s="10" t="n">
-        <v>-52</v>
+        <v>-149</v>
       </c>
       <c r="T13" s="10" t="n">
-        <v>29</v>
+        <v>-43</v>
       </c>
       <c r="U13" s="10" t="n">
-        <v>59</v>
+        <v>-166</v>
       </c>
       <c r="V13" s="10" t="n">
-        <v>-28</v>
+        <v>-413</v>
       </c>
       <c r="W13" s="10" t="n">
-        <v>-98</v>
+        <v>-995</v>
       </c>
       <c r="X13" s="10" t="n">
-        <v>79</v>
+        <v>411</v>
       </c>
       <c r="Y13" s="11" t="n">
-        <v>6</v>
+        <v>-459</v>
       </c>
       <c r="Z13" s="10" t="n">
-        <v>3</v>
+        <v>-321</v>
       </c>
     </row>
     <row r="14">
@@ -1292,79 +1292,79 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="F14" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="O14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="P14" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="R14" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="S14" s="5" t="n">
         <v>69</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>73</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>78</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>84</v>
-      </c>
-      <c r="J14" s="5" t="n">
-        <v>72</v>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>78</v>
-      </c>
-      <c r="L14" s="5" t="n">
-        <v>77</v>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>70</v>
-      </c>
-      <c r="N14" s="5" t="n">
-        <v>87</v>
-      </c>
-      <c r="O14" s="5" t="n">
-        <v>71</v>
-      </c>
-      <c r="P14" s="5" t="n">
-        <v>86</v>
-      </c>
-      <c r="Q14" s="5" t="n">
-        <v>65</v>
-      </c>
-      <c r="R14" s="5" t="n">
-        <v>77</v>
-      </c>
-      <c r="S14" s="5" t="n">
-        <v>72</v>
       </c>
       <c r="T14" s="5" t="n">
         <v>75</v>
       </c>
       <c r="U14" s="5" t="n">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="V14" s="5" t="n">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="W14" s="5" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="X14" s="5" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="Y14" s="12" t="n">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="Z14" s="5" t="n">
-        <v>76</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>